<commit_message>
edit column names, adjust nb to reflect change
</commit_message>
<xml_diff>
--- a/output/test_alt_abbrev_annotation_with_prompt_using_fulltext_and_abstract_df.xlsx
+++ b/output/test_alt_abbrev_annotation_with_prompt_using_fulltext_and_abstract_df.xlsx
@@ -456,57 +456,57 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>captured</t>
+          <t>captured_status</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>captured as:</t>
+          <t>captured_category_list</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>PMIDs from Pubtator3</t>
+          <t>pubtator3_pmid</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Does alias represent gene in this publication?</t>
+          <t>alias_represent_gene_status</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>As an Alternate Abbreviation?</t>
+          <t>alternate_abbreviation_status</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>How? I</t>
+          <t>simple_relationship_type</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>How? II</t>
+          <t>detailed_relationship_type</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>If not this gene, what is it?</t>
+          <t>alias_representation_details</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Text Location</t>
+          <t>relevant_text_section</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Relevant Text (surrounding)</t>
+          <t>relevant_text</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>Notes</t>
+          <t>notes</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
@@ -575,15 +575,11 @@
       <c r="H2" t="n">
         <v>7479945</v>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
+      <c r="I2" t="b">
+        <v>1</v>
+      </c>
+      <c r="J2" t="b">
+        <v>0</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -595,11 +591,7 @@
           <t>mouse phenotype biomarker</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr">
         <is>
           <t>abstract</t>
@@ -661,9 +653,9 @@
     Primary gene symbol: A1CF
     Rules:
     If the text does not support that the alias is an alternate abbreviation, return:
-    "alternate_abbreviation": "NO"
+    "alternate_abbreviation": "FALSE"
     "evidence": ""
-    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
+    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
     Evidence must be one exact sentence copied verbatim from the text.
     Do not infer relationships or paraphrase evidence.
     Output (Strict):
@@ -673,7 +665,7 @@
     "alias_symbol": "",
     "primary_gene_symbol": "",
     "name": "",
-    "alternate_abbreviation": "YES or NO",
+    "alternate_abbreviation": "TRUE or FALSE",
     "evidence": ""
     }
 PMID: 7479945
@@ -687,7 +679,7 @@
 "alias_symbol": "rd5",
 "primary_gene_symbol": "TUB",
 "name": "TUB bipartite transcription factor",
-"alternate_abbreviation": "NO",
+"alternate_abbreviation": "FALSE",
 "evidence": ""
 }</t>
         </is>
@@ -728,15 +720,11 @@
       <c r="H3" t="n">
         <v>9390831</v>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
+      <c r="I3" t="b">
+        <v>1</v>
+      </c>
+      <c r="J3" t="b">
+        <v>0</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -748,11 +736,7 @@
           <t>mouse phenotype biomarker</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr">
         <is>
           <t>abstract</t>
@@ -854,9 +838,9 @@
     Primary gene symbol: A1CF
     Rules:
     If the text does not support that the alias is an alternate abbreviation, return:
-    "alternate_abbreviation": "NO"
+    "alternate_abbreviation": "FALSE"
     "evidence": ""
-    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "YES"
+    If the text does support that the alias is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
     Evidence must be one exact sentence copied verbatim from the text.
     Do not infer relationships or paraphrase evidence.
     Output (Strict):
@@ -866,7 +850,7 @@
     "alias_symbol": "",
     "primary_gene_symbol": "",
     "name": "",
-    "alternate_abbreviation": "YES or NO",
+    "alternate_abbreviation": "TRUE or FALSE",
     "evidence": ""
     }
 PMID: 9390831
@@ -898,7 +882,7 @@
 "alias_symbol": "rd5",
 "primary_gene_symbol": "TUB",
 "name": "TUB bipartite transcription factor",
-"alternate_abbreviation": "NO",
+"alternate_abbreviation": "FALSE",
 "evidence": ""
 }</t>
         </is>

</xml_diff>